<commit_message>
build the endpoints with flasks
</commit_message>
<xml_diff>
--- a/src/report.xlsx
+++ b/src/report.xlsx
@@ -10,6 +10,7 @@
     <sheet name="attendance" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="math" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="automata" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="low level programming" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -7984,6 +7985,3088 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
+      <c r="A1" s="0" t="inlineStr">
+        <is>
+          <t>NAME</t>
+        </is>
+      </c>
+      <c r="B1" s="0" t="inlineStr">
+        <is>
+          <t>INDEX</t>
+        </is>
+      </c>
+      <c r="C1" s="0" t="inlineStr">
+        <is>
+          <t>887:0</t>
+        </is>
+      </c>
+      <c r="D1" s="0" t="inlineStr">
+        <is>
+          <t>461:1</t>
+        </is>
+      </c>
+      <c r="E1" s="0" t="inlineStr">
+        <is>
+          <t>904:2</t>
+        </is>
+      </c>
+      <c r="F1" s="0" t="inlineStr">
+        <is>
+          <t>990:3</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>ADAMS JUNIOR TANK</t>
+        </is>
+      </c>
+      <c r="B2" s="0" t="n">
+        <v>2425403003</v>
+      </c>
+      <c r="C2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>ALAN SITU MESSAN</t>
+        </is>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>2425403755</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="0" t="inlineStr">
+        <is>
+          <t>ALBERT EGHAN</t>
+        </is>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>2425404309</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="0" t="inlineStr">
+        <is>
+          <t>ALEX ANOBI ASARE</t>
+        </is>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>2425402074</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="0" t="inlineStr">
+        <is>
+          <t>ALFRED KWAME NKANSAH AWUKU</t>
+        </is>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>2425402770</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D6" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="0" t="inlineStr">
+        <is>
+          <t>ALVIN TACHIE-MARTIN</t>
+        </is>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>2425402990</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>ANTOINETTE BAIDOO</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="n">
+        <v>2425401488</v>
+      </c>
+      <c r="C8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>ANTOINETTE ENAM AZANU</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="n">
+        <v>2425404665</v>
+      </c>
+      <c r="C9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>BEATRICE DELALI KPEMINI</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="n">
+        <v>2425402514</v>
+      </c>
+      <c r="C10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>BENEDICT ADOFO</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="n">
+        <v>2425403504</v>
+      </c>
+      <c r="C11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="0" t="inlineStr">
+        <is>
+          <t>BENEDICT MARFO KUMI</t>
+        </is>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>2425403210</v>
+      </c>
+      <c r="C12" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="0" t="inlineStr">
+        <is>
+          <t>BENJAMIN YAA-NIETA AMEWU</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>2425402295</v>
+      </c>
+      <c r="C13" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
+          <t>BERNARD ADOTEY KPAKPO</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>2425403899</v>
+      </c>
+      <c r="C14" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>BISMARK KYEI BOATENG</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>2425400268</v>
+      </c>
+      <c r="C15" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
+          <t>BRIGHT OKLU</t>
+        </is>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>2425404334</v>
+      </c>
+      <c r="C16" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="0" t="inlineStr">
+        <is>
+          <t>BRUCE WEGBAH</t>
+        </is>
+      </c>
+      <c r="B17" s="0" t="n">
+        <v>2425400521</v>
+      </c>
+      <c r="C17" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0" t="inlineStr">
+        <is>
+          <t>CALEB KWEKU OKOH</t>
+        </is>
+      </c>
+      <c r="B18" s="0" t="n">
+        <v>2425400891</v>
+      </c>
+      <c r="C18" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0" t="inlineStr">
+        <is>
+          <t>CALEB NII ADJETEY LARYEA</t>
+        </is>
+      </c>
+      <c r="B19" s="0" t="n">
+        <v>2425402475</v>
+      </c>
+      <c r="C19" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0" t="inlineStr">
+        <is>
+          <t>CHRIS ARMAH KOFFIE</t>
+        </is>
+      </c>
+      <c r="B20" s="0" t="n">
+        <v>2425404032</v>
+      </c>
+      <c r="C20" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0" t="inlineStr">
+        <is>
+          <t>CHRIS MAWULORM ADJETEY</t>
+        </is>
+      </c>
+      <c r="B21" s="0" t="n">
+        <v>2425403349</v>
+      </c>
+      <c r="C21" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0" t="inlineStr">
+        <is>
+          <t>CHRISLYN SELASSIE DADIA</t>
+        </is>
+      </c>
+      <c r="B22" s="0" t="n">
+        <v>2425403790</v>
+      </c>
+      <c r="C22" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0" t="inlineStr">
+        <is>
+          <t>CHRISTOPHER NAGETEY</t>
+        </is>
+      </c>
+      <c r="B23" s="0" t="n">
+        <v>2425401676</v>
+      </c>
+      <c r="C23" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>CORNELIUS EDEM TAMAKLOE</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="n">
+        <v>2425400525</v>
+      </c>
+      <c r="C24" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">COURAGE DESMOND AGBO </t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="n">
+        <v>2425401665</v>
+      </c>
+      <c r="C25" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">COURAGE ENOCH TEYE NARTEY </t>
+        </is>
+      </c>
+      <c r="B26" s="0" t="n">
+        <v>2425401317</v>
+      </c>
+      <c r="C26" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0" t="inlineStr">
+        <is>
+          <t>DANIEL ASHIADEY AKAKPO</t>
+        </is>
+      </c>
+      <c r="B27" s="0" t="n">
+        <v>2425404208</v>
+      </c>
+      <c r="C27" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0" t="inlineStr">
+        <is>
+          <t>DANIEL NII AMARH ASHITEY</t>
+        </is>
+      </c>
+      <c r="B28" s="0" t="n">
+        <v>2425402697</v>
+      </c>
+      <c r="C28" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0" t="inlineStr">
+        <is>
+          <t>DARRYL LARBI OTCHERE</t>
+        </is>
+      </c>
+      <c r="B29" s="0" t="n">
+        <v>2425402784</v>
+      </c>
+      <c r="C29" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0" t="inlineStr">
+        <is>
+          <t>DAVID BOAMAH</t>
+        </is>
+      </c>
+      <c r="B30" s="0" t="n">
+        <v>2425403979</v>
+      </c>
+      <c r="C30" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DEBORAH MAMLE ADJOWER </t>
+        </is>
+      </c>
+      <c r="B31" s="0" t="n">
+        <v>2425401764</v>
+      </c>
+      <c r="C31" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0" t="inlineStr">
+        <is>
+          <t>DENNIS DENKYIRA ADU</t>
+        </is>
+      </c>
+      <c r="B32" s="0" t="n">
+        <v>2425403696</v>
+      </c>
+      <c r="C32" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0" t="inlineStr">
+        <is>
+          <t>DONALD KOFFI ANGE AKPAGANA</t>
+        </is>
+      </c>
+      <c r="B33" s="0" t="n">
+        <v>2425404837</v>
+      </c>
+      <c r="C33" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0" t="inlineStr">
+        <is>
+          <t>DORIS KAI ADJEI</t>
+        </is>
+      </c>
+      <c r="B34" s="0" t="n">
+        <v>2425402168</v>
+      </c>
+      <c r="C34" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0" t="inlineStr">
+        <is>
+          <t>DZADZA SHADRACH YAKESSEWA</t>
+        </is>
+      </c>
+      <c r="B35" s="0" t="n">
+        <v>2425400784</v>
+      </c>
+      <c r="C35" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0" t="inlineStr">
+        <is>
+          <t>EDMUND AWUMEY</t>
+        </is>
+      </c>
+      <c r="B36" s="0" t="n">
+        <v>2425403010</v>
+      </c>
+      <c r="C36" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0" t="inlineStr">
+        <is>
+          <t>EDWIN AMPRATWUM</t>
+        </is>
+      </c>
+      <c r="B37" s="0" t="n">
+        <v>2425401458</v>
+      </c>
+      <c r="C37" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0" t="inlineStr">
+        <is>
+          <t>EDWIN DARKO</t>
+        </is>
+      </c>
+      <c r="B38" s="0" t="n">
+        <v>2425401989</v>
+      </c>
+      <c r="C38" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0" t="inlineStr">
+        <is>
+          <t>EKUA BOADUWA MENSAH</t>
+        </is>
+      </c>
+      <c r="B39" s="0" t="n">
+        <v>2425404107</v>
+      </c>
+      <c r="C39" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0" t="inlineStr">
+        <is>
+          <t>ELIJAH TAWIAH DOTSE</t>
+        </is>
+      </c>
+      <c r="B40" s="0" t="n">
+        <v>2425404703</v>
+      </c>
+      <c r="C40" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0" t="inlineStr">
+        <is>
+          <t>ELIZABETH OCANSEY</t>
+        </is>
+      </c>
+      <c r="B41" s="0" t="n">
+        <v>2425401394</v>
+      </c>
+      <c r="C41" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D41" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0" t="inlineStr">
+        <is>
+          <t>EMMANUEL ADOM ESSUMAN</t>
+        </is>
+      </c>
+      <c r="B42" s="0" t="n">
+        <v>2425403347</v>
+      </c>
+      <c r="C42" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E42" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0" t="inlineStr">
+        <is>
+          <t>EMMANUEL AGBEDI</t>
+        </is>
+      </c>
+      <c r="B43" s="0" t="n">
+        <v>2425402768</v>
+      </c>
+      <c r="C43" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0" t="inlineStr">
+        <is>
+          <t>EMMANUEL KWAKYE OSEI</t>
+        </is>
+      </c>
+      <c r="B44" s="0" t="n">
+        <v>2425400974</v>
+      </c>
+      <c r="C44" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E44" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0" t="inlineStr">
+        <is>
+          <t>EMMANUEL NANA KWAME PEPRAH</t>
+        </is>
+      </c>
+      <c r="B45" s="0" t="n">
+        <v>2425401674</v>
+      </c>
+      <c r="C45" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0" t="inlineStr">
+        <is>
+          <t>EMMANUEL OBENG AMOH</t>
+        </is>
+      </c>
+      <c r="B46" s="0" t="n">
+        <v>2425401843</v>
+      </c>
+      <c r="C46" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D46" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0" t="inlineStr">
+        <is>
+          <t>EMMANUEL OWUSU APPIAH ATTAH DWOMOH</t>
+        </is>
+      </c>
+      <c r="B47" s="0" t="n">
+        <v>2425403807</v>
+      </c>
+      <c r="C47" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D47" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0" t="inlineStr">
+        <is>
+          <t>ENOCH KWAME ENNIM BENSON</t>
+        </is>
+      </c>
+      <c r="B48" s="0" t="n">
+        <v>2425400712</v>
+      </c>
+      <c r="C48" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D48" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0" t="inlineStr">
+        <is>
+          <t>ERICA EDEM KANKOE</t>
+        </is>
+      </c>
+      <c r="B49" s="0" t="n">
+        <v>2425401779</v>
+      </c>
+      <c r="C49" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="0" t="inlineStr">
+        <is>
+          <t>ESTHER DIVINA KUENYEHIA</t>
+        </is>
+      </c>
+      <c r="B50" s="0" t="n">
+        <v>2425401137</v>
+      </c>
+      <c r="C50" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D50" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="0" t="inlineStr">
+        <is>
+          <t>EUGENE DELA GOGAH</t>
+        </is>
+      </c>
+      <c r="B51" s="0" t="n">
+        <v>2425402126</v>
+      </c>
+      <c r="C51" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D51" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="0" t="inlineStr">
+        <is>
+          <t>FODJO MATTHEW</t>
+        </is>
+      </c>
+      <c r="B52" s="0" t="n">
+        <v>2425400448</v>
+      </c>
+      <c r="C52" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D52" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F52" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="0" t="inlineStr">
+        <is>
+          <t>FRANK GBENYADE</t>
+        </is>
+      </c>
+      <c r="B53" s="0" t="n">
+        <v>2425401197</v>
+      </c>
+      <c r="C53" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D53" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F53" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="0" t="inlineStr">
+        <is>
+          <t>FRANK NYARKO IBETO UZOR</t>
+        </is>
+      </c>
+      <c r="B54" s="0" t="n">
+        <v>2425402970</v>
+      </c>
+      <c r="C54" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D54" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="0" t="inlineStr">
+        <is>
+          <t>FRANKLYNA DOH-NANI</t>
+        </is>
+      </c>
+      <c r="B55" s="0" t="n">
+        <v>2425404882</v>
+      </c>
+      <c r="C55" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D55" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="0" t="inlineStr">
+        <is>
+          <t>GERALD AGYARE-SIAW</t>
+        </is>
+      </c>
+      <c r="B56" s="0" t="n">
+        <v>2425401157</v>
+      </c>
+      <c r="C56" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D56" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E56" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F56" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="0" t="inlineStr">
+        <is>
+          <t>GERALD OSEI DARKO</t>
+        </is>
+      </c>
+      <c r="B57" s="0" t="n">
+        <v>2425404822</v>
+      </c>
+      <c r="C57" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D57" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F57" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="0" t="inlineStr">
+        <is>
+          <t>GERALD SAMUEL AMPONSAH</t>
+        </is>
+      </c>
+      <c r="B58" s="0" t="n">
+        <v>2425404580</v>
+      </c>
+      <c r="C58" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D58" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E58" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="0" t="inlineStr">
+        <is>
+          <t>GODWIN BOATENG AGYAPONG</t>
+        </is>
+      </c>
+      <c r="B59" s="0" t="n">
+        <v>2425403236</v>
+      </c>
+      <c r="C59" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D59" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E59" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GRACE DUGAH </t>
+        </is>
+      </c>
+      <c r="B60" s="0" t="n">
+        <v>2425400283</v>
+      </c>
+      <c r="C60" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D60" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="0" t="inlineStr">
+        <is>
+          <t>GRAHAM NII TETTEH MENSAH</t>
+        </is>
+      </c>
+      <c r="B61" s="0" t="n">
+        <v>2425403171</v>
+      </c>
+      <c r="C61" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F61" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="0" t="inlineStr">
+        <is>
+          <t>HABEL NARH WORMENOR</t>
+        </is>
+      </c>
+      <c r="B62" s="0" t="n">
+        <v>2425402501</v>
+      </c>
+      <c r="C62" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="0" t="inlineStr">
+        <is>
+          <t>HONESTY YAA BOATEMAA</t>
+        </is>
+      </c>
+      <c r="B63" s="0" t="n">
+        <v>2425402337</v>
+      </c>
+      <c r="C63" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D63" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F63" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="0" t="inlineStr">
+        <is>
+          <t>ISAAC FOSU EFFAH</t>
+        </is>
+      </c>
+      <c r="B64" s="0" t="n">
+        <v>2425403747</v>
+      </c>
+      <c r="C64" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F64" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="0" t="inlineStr">
+        <is>
+          <t>ISIDORE NNAJI NNAMDI</t>
+        </is>
+      </c>
+      <c r="B65" s="0" t="n">
+        <v>2425401135</v>
+      </c>
+      <c r="C65" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D65" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F65" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="0" t="inlineStr">
+        <is>
+          <t>IVAN SEKYI</t>
+        </is>
+      </c>
+      <c r="B66" s="0" t="n">
+        <v>2425403424</v>
+      </c>
+      <c r="C66" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D66" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E66" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="0" t="inlineStr">
+        <is>
+          <t>JACOB TUWOR TETTEH</t>
+        </is>
+      </c>
+      <c r="B67" s="0" t="n">
+        <v>2425402079</v>
+      </c>
+      <c r="C67" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E67" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F67" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="0" t="inlineStr">
+        <is>
+          <t>JAMES WHYTE GYEBI</t>
+        </is>
+      </c>
+      <c r="B68" s="0" t="n">
+        <v>2425401109</v>
+      </c>
+      <c r="C68" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D68" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="0" t="inlineStr">
+        <is>
+          <t>JAMILATU WUNNAM FADLURRAHMAN</t>
+        </is>
+      </c>
+      <c r="B69" s="0" t="n">
+        <v>2425402299</v>
+      </c>
+      <c r="C69" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D69" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E69" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="0" t="inlineStr">
+        <is>
+          <t>JEFFREY ARCHAR</t>
+        </is>
+      </c>
+      <c r="B70" s="0" t="n">
+        <v>2425401298</v>
+      </c>
+      <c r="C70" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E70" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F70" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="0" t="inlineStr">
+        <is>
+          <t>JEFFREY KOOMSON</t>
+        </is>
+      </c>
+      <c r="B71" s="0" t="n">
+        <v>2425401045</v>
+      </c>
+      <c r="C71" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D71" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F71" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="0" t="inlineStr">
+        <is>
+          <t>JEREMIAH BAAH</t>
+        </is>
+      </c>
+      <c r="B72" s="0" t="n">
+        <v>2425403300</v>
+      </c>
+      <c r="C72" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D72" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F72" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="0" t="inlineStr">
+        <is>
+          <t>JEREMY KWABENA APAU LARBI</t>
+        </is>
+      </c>
+      <c r="B73" s="0" t="n">
+        <v>2425401088</v>
+      </c>
+      <c r="C73" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D73" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F73" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="0" t="inlineStr">
+        <is>
+          <t>JERRY NANOR</t>
+        </is>
+      </c>
+      <c r="B74" s="0" t="n">
+        <v>2425402814</v>
+      </c>
+      <c r="C74" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D74" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E74" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F74" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="0" t="inlineStr">
+        <is>
+          <t>JESSIE AVENORGBO</t>
+        </is>
+      </c>
+      <c r="B75" s="0" t="n">
+        <v>2425403719</v>
+      </c>
+      <c r="C75" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D75" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E75" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F75" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="0" t="inlineStr">
+        <is>
+          <t>JOSEPH APELETE BIOSSEY</t>
+        </is>
+      </c>
+      <c r="B76" s="0" t="n">
+        <v>2425401486</v>
+      </c>
+      <c r="C76" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E76" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F76" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="0" t="inlineStr">
+        <is>
+          <t>JOSHUA WILLIAMS</t>
+        </is>
+      </c>
+      <c r="B77" s="0" t="n">
+        <v>2425401231</v>
+      </c>
+      <c r="C77" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D77" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E77" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F77" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="0" t="inlineStr">
+        <is>
+          <t>JUDITH ENYO AFI BLEBOO</t>
+        </is>
+      </c>
+      <c r="B78" s="0" t="n">
+        <v>2425401813</v>
+      </c>
+      <c r="C78" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D78" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E78" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F78" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="0" t="inlineStr">
+        <is>
+          <t>JULIAN AKA ASHONG</t>
+        </is>
+      </c>
+      <c r="B79" s="0" t="n">
+        <v>2425404998</v>
+      </c>
+      <c r="C79" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D79" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E79" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F79" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="0" t="inlineStr">
+        <is>
+          <t>JULIET ESSEL</t>
+        </is>
+      </c>
+      <c r="B80" s="0" t="n">
+        <v>2425402950</v>
+      </c>
+      <c r="C80" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D80" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E80" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F80" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="0" t="inlineStr">
+        <is>
+          <t>JUSTICE NANGUA</t>
+        </is>
+      </c>
+      <c r="B81" s="0" t="n">
+        <v>2425402173</v>
+      </c>
+      <c r="C81" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D81" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E81" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F81" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="0" t="inlineStr">
+        <is>
+          <t>KANYITI RYAN SAFO</t>
+        </is>
+      </c>
+      <c r="B82" s="0" t="n">
+        <v>2425404461</v>
+      </c>
+      <c r="C82" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D82" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E82" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F82" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="0" t="inlineStr">
+        <is>
+          <t>KELVIN AMU</t>
+        </is>
+      </c>
+      <c r="B83" s="0" t="n">
+        <v>2425403579</v>
+      </c>
+      <c r="C83" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D83" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E83" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F83" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="0" t="inlineStr">
+        <is>
+          <t>KELVIN BREMPONG</t>
+        </is>
+      </c>
+      <c r="B84" s="0" t="n">
+        <v>2425403572</v>
+      </c>
+      <c r="C84" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D84" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E84" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F84" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="0" t="inlineStr">
+        <is>
+          <t>KELVIN OBENG KYEREMEH</t>
+        </is>
+      </c>
+      <c r="B85" s="0" t="n">
+        <v>2425403542</v>
+      </c>
+      <c r="C85" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D85" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E85" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F85" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="0" t="inlineStr">
+        <is>
+          <t>KINGSFORD ADU AMPOMAH</t>
+        </is>
+      </c>
+      <c r="B86" s="0" t="n">
+        <v>2425400813</v>
+      </c>
+      <c r="C86" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D86" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E86" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F86" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="0" t="inlineStr">
+        <is>
+          <t>KINGSLEY FOLI AMARKWEI</t>
+        </is>
+      </c>
+      <c r="B87" s="0" t="n">
+        <v>2425404154</v>
+      </c>
+      <c r="C87" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D87" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E87" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F87" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="0" t="inlineStr">
+        <is>
+          <t>KOFI BOATENG SARPONG</t>
+        </is>
+      </c>
+      <c r="B88" s="0" t="n">
+        <v>2425402232</v>
+      </c>
+      <c r="C88" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D88" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E88" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F88" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="0" t="inlineStr">
+        <is>
+          <t>KOFI ODURO BEKOE</t>
+        </is>
+      </c>
+      <c r="B89" s="0" t="n">
+        <v>2425403000</v>
+      </c>
+      <c r="C89" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D89" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E89" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F89" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="0" t="inlineStr">
+        <is>
+          <t>KWABENA BOADU SAFO-BOADI</t>
+        </is>
+      </c>
+      <c r="B90" s="0" t="n">
+        <v>2425402602</v>
+      </c>
+      <c r="C90" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D90" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E90" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F90" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="0" t="inlineStr">
+        <is>
+          <t>KWABENA DARKO OKYERE</t>
+        </is>
+      </c>
+      <c r="B91" s="0" t="n">
+        <v>2425403478</v>
+      </c>
+      <c r="C91" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D91" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E91" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F91" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="0" t="inlineStr">
+        <is>
+          <t>KWABENA NYARKO ABABIO</t>
+        </is>
+      </c>
+      <c r="B92" s="0" t="n">
+        <v>2425400755</v>
+      </c>
+      <c r="C92" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D92" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E92" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F92" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="0" t="inlineStr">
+        <is>
+          <t>KWADWO DAN ANNING</t>
+        </is>
+      </c>
+      <c r="B93" s="0" t="n">
+        <v>2425400903</v>
+      </c>
+      <c r="C93" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D93" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E93" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F93" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="0" t="inlineStr">
+        <is>
+          <t>MACCLEAN KUDOLO</t>
+        </is>
+      </c>
+      <c r="B94" s="0" t="n">
+        <v>2425401291</v>
+      </c>
+      <c r="C94" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D94" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E94" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F94" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="0" t="inlineStr">
+        <is>
+          <t>MARVIN SEAKOMO</t>
+        </is>
+      </c>
+      <c r="B95" s="0" t="n">
+        <v>2425403287</v>
+      </c>
+      <c r="C95" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D95" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E95" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F95" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="0" t="inlineStr">
+        <is>
+          <t>MATHIAS AWUNA AGULASUE</t>
+        </is>
+      </c>
+      <c r="B96" s="0" t="n">
+        <v>2425403737</v>
+      </c>
+      <c r="C96" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D96" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E96" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F96" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="0" t="inlineStr">
+        <is>
+          <t>MAXWELL DUKU</t>
+        </is>
+      </c>
+      <c r="B97" s="0" t="n">
+        <v>2425400296</v>
+      </c>
+      <c r="C97" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D97" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E97" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F97" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="0" t="inlineStr">
+        <is>
+          <t>MICHAEL KWESI BLUDO</t>
+        </is>
+      </c>
+      <c r="B98" s="0" t="n">
+        <v>2425403103</v>
+      </c>
+      <c r="C98" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D98" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E98" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F98" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="0" t="inlineStr">
+        <is>
+          <t>MICHAEL SEYRAM ADZRAKOR</t>
+        </is>
+      </c>
+      <c r="B99" s="0" t="n">
+        <v>2425403047</v>
+      </c>
+      <c r="C99" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D99" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E99" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F99" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="0" t="inlineStr">
+        <is>
+          <t>MOSES QUAYE</t>
+        </is>
+      </c>
+      <c r="B100" s="0" t="n">
+        <v>2425404118</v>
+      </c>
+      <c r="C100" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D100" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E100" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F100" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="0" t="inlineStr">
+        <is>
+          <t>MUHSONAH ABDUL MUGISU</t>
+        </is>
+      </c>
+      <c r="B101" s="0" t="n">
+        <v>2425404171</v>
+      </c>
+      <c r="C101" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D101" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E101" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F101" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="0" t="inlineStr">
+        <is>
+          <t>MUSLIM SEIDU</t>
+        </is>
+      </c>
+      <c r="B102" s="0" t="n">
+        <v>2425402300</v>
+      </c>
+      <c r="C102" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D102" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E102" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F102" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="0" t="inlineStr">
+        <is>
+          <t>NATHANIEL ODONKOR</t>
+        </is>
+      </c>
+      <c r="B103" s="0" t="n">
+        <v>2425404391</v>
+      </c>
+      <c r="C103" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D103" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E103" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F103" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="0" t="inlineStr">
+        <is>
+          <t>NATHANIEL OSEI ASANTE</t>
+        </is>
+      </c>
+      <c r="B104" s="0" t="n">
+        <v>2425402467</v>
+      </c>
+      <c r="C104" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D104" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E104" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F104" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="0" t="inlineStr">
+        <is>
+          <t>NOAH NYARKPO</t>
+        </is>
+      </c>
+      <c r="B105" s="0" t="n">
+        <v>2425402078</v>
+      </c>
+      <c r="C105" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D105" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E105" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F105" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="0" t="inlineStr">
+        <is>
+          <t>OBED YAPKA</t>
+        </is>
+      </c>
+      <c r="B106" s="0" t="n">
+        <v>2425403082</v>
+      </c>
+      <c r="C106" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D106" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E106" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F106" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="0" t="inlineStr">
+        <is>
+          <t>OSCAR NII AKO TETTEH</t>
+        </is>
+      </c>
+      <c r="B107" s="0" t="n">
+        <v>2425402292</v>
+      </c>
+      <c r="C107" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D107" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E107" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F107" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="0" t="inlineStr">
+        <is>
+          <t>PADMON ANTWI ADOMAKO</t>
+        </is>
+      </c>
+      <c r="B108" s="0" t="n">
+        <v>2425402556</v>
+      </c>
+      <c r="C108" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D108" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E108" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F108" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="0" t="inlineStr">
+        <is>
+          <t>PAUL ASARE</t>
+        </is>
+      </c>
+      <c r="B109" s="0" t="n">
+        <v>2425400671</v>
+      </c>
+      <c r="C109" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D109" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E109" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F109" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="0" t="inlineStr">
+        <is>
+          <t>PAUL GWEZEOH KPARDEH</t>
+        </is>
+      </c>
+      <c r="B110" s="0" t="n">
+        <v>2425402792</v>
+      </c>
+      <c r="C110" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D110" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E110" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F110" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="0" t="inlineStr">
+        <is>
+          <t>PHILIP YAW NEEQUAYE ANSAH</t>
+        </is>
+      </c>
+      <c r="B111" s="0" t="n">
+        <v>2425403524</v>
+      </c>
+      <c r="C111" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D111" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E111" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F111" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="0" t="inlineStr">
+        <is>
+          <t>PRINCE LARBI ADDO</t>
+        </is>
+      </c>
+      <c r="B112" s="0" t="n">
+        <v>2425400511</v>
+      </c>
+      <c r="C112" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D112" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E112" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F112" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="0" t="inlineStr">
+        <is>
+          <t>PRINCE SAM QUARCOO</t>
+        </is>
+      </c>
+      <c r="B113" s="0" t="n">
+        <v>2425401107</v>
+      </c>
+      <c r="C113" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D113" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E113" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F113" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="0" t="inlineStr">
+        <is>
+          <t>PRINCE YOUNG DOGBE</t>
+        </is>
+      </c>
+      <c r="B114" s="0" t="n">
+        <v>2425403325</v>
+      </c>
+      <c r="C114" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D114" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E114" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F114" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="0" t="inlineStr">
+        <is>
+          <t>PRINCESS IFEOMA AGBO-ODO</t>
+        </is>
+      </c>
+      <c r="B115" s="0" t="n">
+        <v>2425402739</v>
+      </c>
+      <c r="C115" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D115" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E115" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F115" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="0" t="inlineStr">
+        <is>
+          <t>RAZACK AZIZ</t>
+        </is>
+      </c>
+      <c r="B116" s="0" t="n">
+        <v>2425401771</v>
+      </c>
+      <c r="C116" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D116" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E116" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F116" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="0" t="inlineStr">
+        <is>
+          <t>REBECCA TACKIE</t>
+        </is>
+      </c>
+      <c r="B117" s="0" t="n">
+        <v>2425402180</v>
+      </c>
+      <c r="C117" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D117" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E117" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F117" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="0" t="inlineStr">
+        <is>
+          <t>RICHMOND ASANTE</t>
+        </is>
+      </c>
+      <c r="B118" s="0" t="n">
+        <v>2425403688</v>
+      </c>
+      <c r="C118" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D118" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E118" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F118" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="0" t="inlineStr">
+        <is>
+          <t>ROSEMARY AWOENAM YEVOO</t>
+        </is>
+      </c>
+      <c r="B119" s="0" t="n">
+        <v>2425402524</v>
+      </c>
+      <c r="C119" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D119" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E119" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F119" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="0" t="inlineStr">
+        <is>
+          <t>RUBEN OFORI ESHUN</t>
+        </is>
+      </c>
+      <c r="B120" s="0" t="n">
+        <v>2425404102</v>
+      </c>
+      <c r="C120" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D120" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E120" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F120" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="0" t="inlineStr">
+        <is>
+          <t>RUTH TESSU</t>
+        </is>
+      </c>
+      <c r="B121" s="0" t="n">
+        <v>2425404251</v>
+      </c>
+      <c r="C121" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D121" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E121" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F121" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="0" t="inlineStr">
+        <is>
+          <t>SALIU ISSAKA</t>
+        </is>
+      </c>
+      <c r="B122" s="0" t="n">
+        <v>2425402813</v>
+      </c>
+      <c r="C122" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D122" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E122" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F122" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="0" t="inlineStr">
+        <is>
+          <t>SAMUEL AMO ADJEI</t>
+        </is>
+      </c>
+      <c r="B123" s="0" t="n">
+        <v>2425400321</v>
+      </c>
+      <c r="C123" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D123" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E123" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F123" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="0" t="inlineStr">
+        <is>
+          <t>SAMUEL ASEDA QUARTSON</t>
+        </is>
+      </c>
+      <c r="B124" s="0" t="n">
+        <v>2425400839</v>
+      </c>
+      <c r="C124" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D124" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E124" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F124" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="0" t="inlineStr">
+        <is>
+          <t>SAMUEL OBENG APPIAH-KUBI</t>
+        </is>
+      </c>
+      <c r="B125" s="0" t="n">
+        <v>2425401187</v>
+      </c>
+      <c r="C125" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D125" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E125" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F125" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="0" t="inlineStr">
+        <is>
+          <t>SAMUEL YAW POBEE</t>
+        </is>
+      </c>
+      <c r="B126" s="0" t="n">
+        <v>2425404428</v>
+      </c>
+      <c r="C126" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D126" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E126" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F126" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="0" t="inlineStr">
+        <is>
+          <t>SELORM KWABENA KAMASA</t>
+        </is>
+      </c>
+      <c r="B127" s="0" t="n">
+        <v>2425403176</v>
+      </c>
+      <c r="C127" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D127" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E127" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F127" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="0" t="inlineStr">
+        <is>
+          <t>SERENE KLENAM  MENSAH</t>
+        </is>
+      </c>
+      <c r="B128" s="0" t="n">
+        <v>2425400997</v>
+      </c>
+      <c r="C128" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D128" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E128" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F128" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="0" t="inlineStr">
+        <is>
+          <t>STEPHEN KOFI GADZEY</t>
+        </is>
+      </c>
+      <c r="B129" s="0" t="n">
+        <v>2425403282</v>
+      </c>
+      <c r="C129" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D129" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E129" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F129" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="0" t="inlineStr">
+        <is>
+          <t>SUSANNA NANA AKUA AKYIAA AMOAKO</t>
+        </is>
+      </c>
+      <c r="B130" s="0" t="n">
+        <v>2425400613</v>
+      </c>
+      <c r="C130" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D130" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E130" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F130" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SYLVESTER AGYIRI </t>
+        </is>
+      </c>
+      <c r="B131" s="0" t="n">
+        <v>2425402862</v>
+      </c>
+      <c r="C131" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D131" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E131" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F131" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="0" t="inlineStr">
+        <is>
+          <t>TAHOFEEQ JAMIU</t>
+        </is>
+      </c>
+      <c r="B132" s="0" t="n">
+        <v>2425403114</v>
+      </c>
+      <c r="C132" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D132" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E132" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F132" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="0" t="inlineStr">
+        <is>
+          <t>THEOPHILUS MAWUKO SEWORNU</t>
+        </is>
+      </c>
+      <c r="B133" s="0" t="n">
+        <v>2425400343</v>
+      </c>
+      <c r="C133" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D133" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E133" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F133" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="0" t="inlineStr">
+        <is>
+          <t>THEOPHILUS OSEI BONSU</t>
+        </is>
+      </c>
+      <c r="B134" s="0" t="n">
+        <v>2425403196</v>
+      </c>
+      <c r="C134" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D134" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E134" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F134" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="0" t="inlineStr">
+        <is>
+          <t>THOMPSON BOATENG AMPONSAH</t>
+        </is>
+      </c>
+      <c r="B135" s="0" t="n">
+        <v>2425401059</v>
+      </c>
+      <c r="C135" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D135" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E135" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F135" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="0" t="inlineStr">
+        <is>
+          <t>TRACY OHEMAA YAA BOATENG</t>
+        </is>
+      </c>
+      <c r="B136" s="0" t="n">
+        <v>2425402105</v>
+      </c>
+      <c r="C136" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D136" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E136" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="F136" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UBEYDAH YUSSUF </t>
+        </is>
+      </c>
+      <c r="B137" s="0" t="n">
+        <v>2425403965</v>
+      </c>
+      <c r="C137" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D137" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E137" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F137" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="0" t="inlineStr">
+        <is>
+          <t>VERONICA SERWAH BOATENG</t>
+        </is>
+      </c>
+      <c r="B138" s="0" t="n">
+        <v>2425400543</v>
+      </c>
+      <c r="C138" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D138" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="E138" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F138" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="0" t="inlineStr">
+        <is>
+          <t>VICTOR URIEL NII LARYEA DOKU</t>
+        </is>
+      </c>
+      <c r="B139" s="0" t="n">
+        <v>2425402390</v>
+      </c>
+      <c r="C139" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="D139" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E139" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F139" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E139"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
       <c r="A1" t="inlineStr">
         <is>
           <t>NAME</t>
@@ -8007,11 +11090,6 @@
       <c r="E1" t="inlineStr">
         <is>
           <t>904:2</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>990:3</t>
         </is>
       </c>
     </row>
@@ -8033,9 +11111,6 @@
       <c r="E2" t="n">
         <v>0</v>
       </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -8055,9 +11130,6 @@
       <c r="E3" t="n">
         <v>0</v>
       </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -8077,9 +11149,6 @@
       <c r="E4" t="n">
         <v>1</v>
       </c>
-      <c r="F4" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -8099,9 +11168,6 @@
       <c r="E5" t="n">
         <v>1</v>
       </c>
-      <c r="F5" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -8121,9 +11187,6 @@
       <c r="E6" t="n">
         <v>1</v>
       </c>
-      <c r="F6" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -8143,9 +11206,6 @@
       <c r="E7" t="n">
         <v>0</v>
       </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -8165,9 +11225,6 @@
       <c r="E8" t="n">
         <v>1</v>
       </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -8187,9 +11244,6 @@
       <c r="E9" t="n">
         <v>1</v>
       </c>
-      <c r="F9" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -8209,9 +11263,6 @@
       <c r="E10" t="n">
         <v>1</v>
       </c>
-      <c r="F10" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -8231,9 +11282,6 @@
       <c r="E11" t="n">
         <v>1</v>
       </c>
-      <c r="F11" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -8253,9 +11301,6 @@
       <c r="E12" t="n">
         <v>1</v>
       </c>
-      <c r="F12" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -8275,9 +11320,6 @@
       <c r="E13" t="n">
         <v>1</v>
       </c>
-      <c r="F13" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -8297,9 +11339,6 @@
       <c r="E14" t="n">
         <v>1</v>
       </c>
-      <c r="F14" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -8319,9 +11358,6 @@
       <c r="E15" t="n">
         <v>1</v>
       </c>
-      <c r="F15" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -8341,9 +11377,6 @@
       <c r="E16" t="n">
         <v>1</v>
       </c>
-      <c r="F16" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -8363,9 +11396,6 @@
       <c r="E17" t="n">
         <v>1</v>
       </c>
-      <c r="F17" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -8385,9 +11415,6 @@
       <c r="E18" t="n">
         <v>1</v>
       </c>
-      <c r="F18" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -8407,9 +11434,6 @@
       <c r="E19" t="n">
         <v>0</v>
       </c>
-      <c r="F19" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -8429,9 +11453,6 @@
       <c r="E20" t="n">
         <v>1</v>
       </c>
-      <c r="F20" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -8451,9 +11472,6 @@
       <c r="E21" t="n">
         <v>1</v>
       </c>
-      <c r="F21" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -8473,9 +11491,6 @@
       <c r="E22" t="n">
         <v>0</v>
       </c>
-      <c r="F22" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -8495,9 +11510,6 @@
       <c r="E23" t="n">
         <v>0</v>
       </c>
-      <c r="F23" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -8517,9 +11529,6 @@
       <c r="E24" t="n">
         <v>0</v>
       </c>
-      <c r="F24" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -8539,9 +11548,6 @@
       <c r="E25" t="n">
         <v>1</v>
       </c>
-      <c r="F25" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -8561,9 +11567,6 @@
       <c r="E26" t="n">
         <v>1</v>
       </c>
-      <c r="F26" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -8583,9 +11586,6 @@
       <c r="E27" t="n">
         <v>0</v>
       </c>
-      <c r="F27" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -8605,9 +11605,6 @@
       <c r="E28" t="n">
         <v>1</v>
       </c>
-      <c r="F28" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -8627,9 +11624,6 @@
       <c r="E29" t="n">
         <v>1</v>
       </c>
-      <c r="F29" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -8649,9 +11643,6 @@
       <c r="E30" t="n">
         <v>1</v>
       </c>
-      <c r="F30" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -8671,9 +11662,6 @@
       <c r="E31" t="n">
         <v>1</v>
       </c>
-      <c r="F31" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -8693,9 +11681,6 @@
       <c r="E32" t="n">
         <v>1</v>
       </c>
-      <c r="F32" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -8715,9 +11700,6 @@
       <c r="E33" t="n">
         <v>0</v>
       </c>
-      <c r="F33" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -8737,9 +11719,6 @@
       <c r="E34" t="n">
         <v>1</v>
       </c>
-      <c r="F34" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -8759,9 +11738,6 @@
       <c r="E35" t="n">
         <v>1</v>
       </c>
-      <c r="F35" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -8781,9 +11757,6 @@
       <c r="E36" t="n">
         <v>1</v>
       </c>
-      <c r="F36" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -8803,9 +11776,6 @@
       <c r="E37" t="n">
         <v>1</v>
       </c>
-      <c r="F37" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -8825,9 +11795,6 @@
       <c r="E38" t="n">
         <v>0</v>
       </c>
-      <c r="F38" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8847,9 +11814,6 @@
       <c r="E39" t="n">
         <v>0</v>
       </c>
-      <c r="F39" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -8869,9 +11833,6 @@
       <c r="E40" t="n">
         <v>0</v>
       </c>
-      <c r="F40" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -8891,9 +11852,6 @@
       <c r="E41" t="n">
         <v>1</v>
       </c>
-      <c r="F41" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -8913,9 +11871,6 @@
       <c r="E42" t="n">
         <v>1</v>
       </c>
-      <c r="F42" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -8935,9 +11890,6 @@
       <c r="E43" t="n">
         <v>1</v>
       </c>
-      <c r="F43" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -8957,9 +11909,6 @@
       <c r="E44" t="n">
         <v>1</v>
       </c>
-      <c r="F44" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -8979,9 +11928,6 @@
       <c r="E45" t="n">
         <v>0</v>
       </c>
-      <c r="F45" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -9001,9 +11947,6 @@
       <c r="E46" t="n">
         <v>1</v>
       </c>
-      <c r="F46" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -9023,9 +11966,6 @@
       <c r="E47" t="n">
         <v>0</v>
       </c>
-      <c r="F47" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -9045,9 +11985,6 @@
       <c r="E48" t="n">
         <v>0</v>
       </c>
-      <c r="F48" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -9067,9 +12004,6 @@
       <c r="E49" t="n">
         <v>0</v>
       </c>
-      <c r="F49" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -9089,9 +12023,6 @@
       <c r="E50" t="n">
         <v>1</v>
       </c>
-      <c r="F50" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -9111,9 +12042,6 @@
       <c r="E51" t="n">
         <v>1</v>
       </c>
-      <c r="F51" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -9133,9 +12061,6 @@
       <c r="E52" t="n">
         <v>1</v>
       </c>
-      <c r="F52" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -9155,9 +12080,6 @@
       <c r="E53" t="n">
         <v>0</v>
       </c>
-      <c r="F53" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -9177,9 +12099,6 @@
       <c r="E54" t="n">
         <v>1</v>
       </c>
-      <c r="F54" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -9199,9 +12118,6 @@
       <c r="E55" t="n">
         <v>1</v>
       </c>
-      <c r="F55" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -9221,9 +12137,6 @@
       <c r="E56" t="n">
         <v>1</v>
       </c>
-      <c r="F56" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -9243,9 +12156,6 @@
       <c r="E57" t="n">
         <v>0</v>
       </c>
-      <c r="F57" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -9265,9 +12175,6 @@
       <c r="E58" t="n">
         <v>1</v>
       </c>
-      <c r="F58" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -9287,9 +12194,6 @@
       <c r="E59" t="n">
         <v>1</v>
       </c>
-      <c r="F59" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -9309,9 +12213,6 @@
       <c r="E60" t="n">
         <v>1</v>
       </c>
-      <c r="F60" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -9331,9 +12232,6 @@
       <c r="E61" t="n">
         <v>1</v>
       </c>
-      <c r="F61" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -9353,9 +12251,6 @@
       <c r="E62" t="n">
         <v>1</v>
       </c>
-      <c r="F62" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -9375,9 +12270,6 @@
       <c r="E63" t="n">
         <v>1</v>
       </c>
-      <c r="F63" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -9397,9 +12289,6 @@
       <c r="E64" t="n">
         <v>1</v>
       </c>
-      <c r="F64" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -9419,9 +12308,6 @@
       <c r="E65" t="n">
         <v>1</v>
       </c>
-      <c r="F65" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -9441,9 +12327,6 @@
       <c r="E66" t="n">
         <v>1</v>
       </c>
-      <c r="F66" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -9463,9 +12346,6 @@
       <c r="E67" t="n">
         <v>0</v>
       </c>
-      <c r="F67" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -9485,9 +12365,6 @@
       <c r="E68" t="n">
         <v>1</v>
       </c>
-      <c r="F68" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -9507,9 +12384,6 @@
       <c r="E69" t="n">
         <v>1</v>
       </c>
-      <c r="F69" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -9529,9 +12403,6 @@
       <c r="E70" t="n">
         <v>1</v>
       </c>
-      <c r="F70" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -9551,9 +12422,6 @@
       <c r="E71" t="n">
         <v>1</v>
       </c>
-      <c r="F71" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -9573,9 +12441,6 @@
       <c r="E72" t="n">
         <v>0</v>
       </c>
-      <c r="F72" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -9595,9 +12460,6 @@
       <c r="E73" t="n">
         <v>1</v>
       </c>
-      <c r="F73" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -9617,9 +12479,6 @@
       <c r="E74" t="n">
         <v>0</v>
       </c>
-      <c r="F74" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -9639,9 +12498,6 @@
       <c r="E75" t="n">
         <v>0</v>
       </c>
-      <c r="F75" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -9661,9 +12517,6 @@
       <c r="E76" t="n">
         <v>1</v>
       </c>
-      <c r="F76" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -9683,9 +12536,6 @@
       <c r="E77" t="n">
         <v>0</v>
       </c>
-      <c r="F77" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -9705,9 +12555,6 @@
       <c r="E78" t="n">
         <v>1</v>
       </c>
-      <c r="F78" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -9727,9 +12574,6 @@
       <c r="E79" t="n">
         <v>1</v>
       </c>
-      <c r="F79" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -9749,9 +12593,6 @@
       <c r="E80" t="n">
         <v>0</v>
       </c>
-      <c r="F80" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -9771,9 +12612,6 @@
       <c r="E81" t="n">
         <v>1</v>
       </c>
-      <c r="F81" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -9793,9 +12631,6 @@
       <c r="E82" t="n">
         <v>1</v>
       </c>
-      <c r="F82" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -9815,9 +12650,6 @@
       <c r="E83" t="n">
         <v>1</v>
       </c>
-      <c r="F83" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -9837,9 +12669,6 @@
       <c r="E84" t="n">
         <v>1</v>
       </c>
-      <c r="F84" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -9859,9 +12688,6 @@
       <c r="E85" t="n">
         <v>1</v>
       </c>
-      <c r="F85" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -9881,9 +12707,6 @@
       <c r="E86" t="n">
         <v>1</v>
       </c>
-      <c r="F86" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -9903,9 +12726,6 @@
       <c r="E87" t="n">
         <v>1</v>
       </c>
-      <c r="F87" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -9925,9 +12745,6 @@
       <c r="E88" t="n">
         <v>0</v>
       </c>
-      <c r="F88" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -9947,9 +12764,6 @@
       <c r="E89" t="n">
         <v>0</v>
       </c>
-      <c r="F89" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -9969,9 +12783,6 @@
       <c r="E90" t="n">
         <v>1</v>
       </c>
-      <c r="F90" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -9991,9 +12802,6 @@
       <c r="E91" t="n">
         <v>0</v>
       </c>
-      <c r="F91" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -10013,9 +12821,6 @@
       <c r="E92" t="n">
         <v>1</v>
       </c>
-      <c r="F92" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -10035,9 +12840,6 @@
       <c r="E93" t="n">
         <v>1</v>
       </c>
-      <c r="F93" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -10057,9 +12859,6 @@
       <c r="E94" t="n">
         <v>1</v>
       </c>
-      <c r="F94" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -10079,9 +12878,6 @@
       <c r="E95" t="n">
         <v>1</v>
       </c>
-      <c r="F95" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -10101,9 +12897,6 @@
       <c r="E96" t="n">
         <v>0</v>
       </c>
-      <c r="F96" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -10123,9 +12916,6 @@
       <c r="E97" t="n">
         <v>1</v>
       </c>
-      <c r="F97" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -10145,9 +12935,6 @@
       <c r="E98" t="n">
         <v>0</v>
       </c>
-      <c r="F98" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -10167,9 +12954,6 @@
       <c r="E99" t="n">
         <v>1</v>
       </c>
-      <c r="F99" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -10189,9 +12973,6 @@
       <c r="E100" t="n">
         <v>1</v>
       </c>
-      <c r="F100" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -10211,9 +12992,6 @@
       <c r="E101" t="n">
         <v>1</v>
       </c>
-      <c r="F101" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -10233,9 +13011,6 @@
       <c r="E102" t="n">
         <v>1</v>
       </c>
-      <c r="F102" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -10255,9 +13030,6 @@
       <c r="E103" t="n">
         <v>1</v>
       </c>
-      <c r="F103" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -10277,9 +13049,6 @@
       <c r="E104" t="n">
         <v>1</v>
       </c>
-      <c r="F104" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -10299,9 +13068,6 @@
       <c r="E105" t="n">
         <v>1</v>
       </c>
-      <c r="F105" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -10321,9 +13087,6 @@
       <c r="E106" t="n">
         <v>1</v>
       </c>
-      <c r="F106" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -10343,9 +13106,6 @@
       <c r="E107" t="n">
         <v>1</v>
       </c>
-      <c r="F107" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -10365,9 +13125,6 @@
       <c r="E108" t="n">
         <v>1</v>
       </c>
-      <c r="F108" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -10387,9 +13144,6 @@
       <c r="E109" t="n">
         <v>1</v>
       </c>
-      <c r="F109" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -10409,9 +13163,6 @@
       <c r="E110" t="n">
         <v>0</v>
       </c>
-      <c r="F110" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -10431,9 +13182,6 @@
       <c r="E111" t="n">
         <v>0</v>
       </c>
-      <c r="F111" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -10453,9 +13201,6 @@
       <c r="E112" t="n">
         <v>1</v>
       </c>
-      <c r="F112" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -10475,9 +13220,6 @@
       <c r="E113" t="n">
         <v>1</v>
       </c>
-      <c r="F113" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -10497,9 +13239,6 @@
       <c r="E114" t="n">
         <v>1</v>
       </c>
-      <c r="F114" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -10519,9 +13258,6 @@
       <c r="E115" t="n">
         <v>0</v>
       </c>
-      <c r="F115" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -10541,9 +13277,6 @@
       <c r="E116" t="n">
         <v>0</v>
       </c>
-      <c r="F116" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -10563,9 +13296,6 @@
       <c r="E117" t="n">
         <v>0</v>
       </c>
-      <c r="F117" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -10585,9 +13315,6 @@
       <c r="E118" t="n">
         <v>1</v>
       </c>
-      <c r="F118" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -10607,9 +13334,6 @@
       <c r="E119" t="n">
         <v>1</v>
       </c>
-      <c r="F119" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -10629,9 +13353,6 @@
       <c r="E120" t="n">
         <v>0</v>
       </c>
-      <c r="F120" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -10651,9 +13372,6 @@
       <c r="E121" t="n">
         <v>1</v>
       </c>
-      <c r="F121" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -10673,9 +13391,6 @@
       <c r="E122" t="n">
         <v>0</v>
       </c>
-      <c r="F122" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -10695,9 +13410,6 @@
       <c r="E123" t="n">
         <v>1</v>
       </c>
-      <c r="F123" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -10717,9 +13429,6 @@
       <c r="E124" t="n">
         <v>0</v>
       </c>
-      <c r="F124" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -10739,9 +13448,6 @@
       <c r="E125" t="n">
         <v>0</v>
       </c>
-      <c r="F125" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -10761,9 +13467,6 @@
       <c r="E126" t="n">
         <v>1</v>
       </c>
-      <c r="F126" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -10783,9 +13486,6 @@
       <c r="E127" t="n">
         <v>1</v>
       </c>
-      <c r="F127" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -10805,9 +13505,6 @@
       <c r="E128" t="n">
         <v>1</v>
       </c>
-      <c r="F128" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -10827,9 +13524,6 @@
       <c r="E129" t="n">
         <v>0</v>
       </c>
-      <c r="F129" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -10849,9 +13543,6 @@
       <c r="E130" t="n">
         <v>0</v>
       </c>
-      <c r="F130" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -10871,9 +13562,6 @@
       <c r="E131" t="n">
         <v>0</v>
       </c>
-      <c r="F131" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -10893,9 +13581,6 @@
       <c r="E132" t="n">
         <v>0</v>
       </c>
-      <c r="F132" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -10915,9 +13600,6 @@
       <c r="E133" t="n">
         <v>1</v>
       </c>
-      <c r="F133" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -10937,9 +13619,6 @@
       <c r="E134" t="n">
         <v>0</v>
       </c>
-      <c r="F134" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -10959,9 +13638,6 @@
       <c r="E135" t="n">
         <v>1</v>
       </c>
-      <c r="F135" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -10981,9 +13657,6 @@
       <c r="E136" t="n">
         <v>0</v>
       </c>
-      <c r="F136" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -11003,9 +13676,6 @@
       <c r="E137" t="n">
         <v>1</v>
       </c>
-      <c r="F137" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -11025,9 +13695,6 @@
       <c r="E138" t="n">
         <v>1</v>
       </c>
-      <c r="F138" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -11045,9 +13712,6 @@
         <v>1</v>
       </c>
       <c r="E139" t="n">
-        <v>1</v>
-      </c>
-      <c r="F139" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>